<commit_message>
form input & update approvals
</commit_message>
<xml_diff>
--- a/merged_current.xlsx
+++ b/merged_current.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R105"/>
+  <dimension ref="A1:R155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,7 +584,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Director B</t>
+          <t>admin</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Director B</t>
+          <t>NOP-PALU</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Director B</t>
+          <t>NOP-PALU</t>
         </is>
       </c>
     </row>
@@ -9669,6 +9669,4406 @@
       <c r="R105" t="inlineStr">
         <is>
           <t>COO - Sinta Maharani</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>NOP-2001</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Brand Awareness Campaign</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-1 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 1</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>30171196</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>46493805</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>21013562</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>25480243</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>5244582</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>6216546</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>10520896</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>NOP-2002</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-2 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 2</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>34051036</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>56419230</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>20698440</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>35720790</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>5632675</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>6654931</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>13062812</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>NOP-2003</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Service Improvement</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-3 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 3</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>44039922</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>86135703</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>31236714</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>54898989</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>4453055</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>15271403</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>19890806</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>NOP-2004</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-4 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 4</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>40455600</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>71925028</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>32013276</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>39911752</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>6918158</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>10790444</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>11919572</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>NOP-2005</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-5 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 5</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>36401370</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>69351043</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>24064386</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>45286658</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>3720250</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>11978462</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>16974241</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>NOP-2006</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Service Improvement</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-6 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 6</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>21817601</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>40006729</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>15864256</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>24142473</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>4733712</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>6258036</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>7370060</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>NOP-2007</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Brand Awareness Campaign</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-7 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 7</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>72899870</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>129466977</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>53597448</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>75869529</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>8212187</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>15572051</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>21879036</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>NOP-2008</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-8 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 8</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>63952509</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>94104923</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>49785072</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>44319851</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>11200382</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>10312490</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>15266908</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>NOP-2009</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-9 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 9</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>54241738</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>102829636</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>38478122</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>64351514</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>7266845</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>14736395</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>15798931</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>NOP-2010</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Market Expansion</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-10 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 10</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>40578628</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>67012630</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>28967477</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>38045153</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>7631340</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>11908725</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>10203015</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>NOP-2011</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Market Expansion</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-11 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 11</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>64709008</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>84873002</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>47407259</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>37465742</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>8969554</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>11499719</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>13512675</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>NOP-2012</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-12 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 12</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>23968407</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>38836545</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>17842735</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>20993811</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>3323778</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>5307560</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>6388816</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>NOP-2013</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-13 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 13</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>68429648</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>118671775</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>55771767</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>62900008</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>13122193</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>14956217</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>28559625</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>NOP-2014</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Market Expansion</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-14 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 14</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>45532805</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>79740288</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>30292063</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>49448225</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>4316776</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>7981897</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>17929197</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>NOP-2015</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Market Expansion</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-15 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 15</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>23485533</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>33567781</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>17182807</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>16384974</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>2426161</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>5574954</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>7425696</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>NOP-2016</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Brand Awareness Campaign</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-16 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 16</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>73636801</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>122925764</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>59311569</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>63614195</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>6735931</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>18121808</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>29234191</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>NOP-2017</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Market Expansion</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-17 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 17</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>52893218</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>78544217</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>39574997</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>38969220</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>8389633</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>13605713</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>19633618</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>NOP-2018</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Service Improvement</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-18 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 18</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>65821144</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>126211846</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>43108494</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>83103352</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>12609940</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>14637573</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>25698670</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>NOP-2019</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Brand Awareness Campaign</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-19 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 19</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>29533958</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>47071075</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>24576652</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>22494423</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>4562010</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>5984649</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>11124868</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>NOP-2020</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-20 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 20</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>49774406</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>78437403</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>31478217</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>46959185</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>8181732</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>13620420</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>18062662</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>NOP-2021</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Service Improvement</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-21 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 21</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>42980873</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>74524912</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>31752499</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>42772413</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>6577961</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>10972609</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>14497824</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>NOP-2022</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-22 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 22</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>36338601</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>60810962</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>22918832</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>37892130</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>6846532</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>10248724</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>12926334</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>NOP-2023</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Brand Awareness Campaign</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-23 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 23</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>37907837</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>63966186</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>29464572</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>34501615</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>5318612</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>11228199</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>14831118</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>NOP-2024</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-24 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 24</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>30896616</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>56891933</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>19003146</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>37888787</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>5425301</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>9069712</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>11331287</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>NOP-2025</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Service Improvement</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-25 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 25</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>39919495</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>57001751</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>25759829</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>31241923</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>3551907</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>9990450</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>12580015</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>NOP-2026</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Market Expansion</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-26 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 26</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>42034925</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>80748870</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>33063224</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>47685647</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>5198971</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>12434652</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>19053909</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>NOP-2027</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-27 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 27</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>59196820</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>94040062</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>49398702</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>44641359</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>6851166</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>10348889</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>14370476</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>NOP-2028</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Brand Awareness Campaign</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-28 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 28</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>29740842</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>61279458</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>24096771</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>37182687</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>6673074</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>9031332</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>10048378</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>NOP-2029</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Brand Awareness Campaign</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-29 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 29</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>15777278</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>29823768</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>11530735</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>18293032</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>3424404</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>4626255</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>6352308</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>NOP-2030</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-30 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 30</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>64175422</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>93093983</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>45623482</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>47470501</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>11035077</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>15445494</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>22835106</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>NOP-2031</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-31 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 31</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>74369323</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>111231094</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>55321384</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>55909709</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>5624766</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>17547838</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>18674308</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>NOP-2032</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Market Expansion</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-32 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 32</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>37892649</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>74183759</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>25273360</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>48910398</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>8812046</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>7609017</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>12353750</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>NOP-2033</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-33 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 33</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>40944755</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>80900731</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>32413955</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>48486776</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>7576025</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>9999620</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>19987818</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>NOP-2034</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-34 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 34</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>24635592</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>50060057</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>20907232</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>29152825</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>3710659</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>8667631</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>11411519</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>NOP-2035</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-35 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 35</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>15455240</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>29660129</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>11812897</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>17847231</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>2618109</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>4824422</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>4950272</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>NOP-2036</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Service Improvement</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-36 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 36</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>66675079</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>104263013</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>50854079</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>53408933</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>5282976</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>15869937</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>19317986</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>NOP-2037</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Service Improvement</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-37 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 37</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>25569061</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>43446007</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>17509657</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>25936350</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>4202747</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>7009234</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>7917843</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>NOP-2038</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Service Improvement</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-38 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 38</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>48030882</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>94669089</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>36191167</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>58477922</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>10097016</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>11293264</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>23454059</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>NOP-2039</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-39 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 39</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>45759545</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>78881023</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>38308676</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>40572347</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>4423493</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>11953896</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>13779443</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>NOP-2040</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Brand Awareness Campaign</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-40 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 40</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>43970234</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>64863743</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>30099190</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>34764553</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>5699460</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>9353733</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>12863486</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>NOP-2041</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Service Improvement</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-41 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 41</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>38272133</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>55419444</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>23152837</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>32266607</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>2885508</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>5708445</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>8722052</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>NOP-2042</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-42 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 42</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>34757676</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>48821347</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>23992090</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>24829257</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>3046141</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>5507973</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>9252879</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>Lead C</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>NOP-2043</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-43 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 43</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>23893557</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>39891462</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>15576320</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>24315142</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>2121770</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>4252607</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>8157283</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>NOP-2044</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-44 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 44</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>71431265</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>113833612</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>60553655</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>53279957</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>7878979</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>11918781</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>23313287</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>Technology Division</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>NOP-2045</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-45 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 45</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>61667593</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>84978333</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>49124416</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>35853917</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>8893099</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>8623876</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>17898908</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>NOP-2046</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-46 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 46</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>25601558</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>38570449</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>17568632</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>21001817</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>1966915</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>4020260</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>7289724</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>NOP-2047</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-47 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 47</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>51282409</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>68487479</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>37031004</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>31456476</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>7272042</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>11053667</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>12549437</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>NOP-2048</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Brand Awareness Campaign</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-48 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 48</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>67678105</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>102720718</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>57519124</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>45201594</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>7131892</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>15172410</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>22718126</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>Lead A</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>NOP-2049</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Process Automation</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-49 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 49</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>58825117</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>107886974</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>37988364</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>69898610</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>6917097</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>13523516</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>19221975</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>VP Y</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>VP X</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>NOP-2050</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Data Analytics Initiative</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Justifikasi inisiatif bisnis ke-50 untuk peningkatan revenue</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Proposal Inisiatif 50</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>40165768</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>73363373</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>33206543</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>40156829</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>4262039</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>9648369</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>17798416</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>Lead B</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>VP X</t>
         </is>
       </c>
     </row>

</xml_diff>